<commit_message>
feat: implement LLM field resolution and usage reconciliation pipeline with comprehensive testing and evaluation reports
</commit_message>
<xml_diff>
--- a/gold_standard/tenders/GAIL Visakhapatnam B&BC VRLA_InfoSheet.xlsx
+++ b/gold_standard/tenders/GAIL Visakhapatnam B&BC VRLA_InfoSheet.xlsx
@@ -205,9 +205,6 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -217,7 +214,7 @@
     <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -240,6 +237,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -627,14 +627,14 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Total Schema Fields: 95  |  OK (Extracted): 59  |  OK (Fallback): 0  |  N/A (Not Applicable): 17  |  ⚠️ MISSING: 19</t>
+          <t>Total Schema Fields: 95  |  OK (Extracted): 62  |  OK (Fallback): 0  |  N/A (Not Applicable): 25  |  ⚠️ MISSING: 8</t>
         </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>⚠️ ACTION REQUIRED — Missing Fields (19): Website, Te Recommendation, Processing Fee Mode, Tender Fee Mode, Tender Value, Sd Duration, Order Value 1, Order Value 2 (+11 more)</t>
+          <t>⚠️ ACTION REQUIRED — Missing Fields (8): Client Phone 1, Client Phone 2, Courier Provider, Courier Docket No, Courier Delivery Time, Docket Slip Upload, Physical Docs Uploaded, Schedule 4 Details</t>
         </is>
       </c>
     </row>
@@ -660,7 +660,7 @@
       <c r="B6" s="5" t="n"/>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Not mandatory / Self-acquaintance (Bidder advised to inspect site before bidding)</t>
+          <t>No / Self-Certification (Deemed site visit acknowledgment in SCC; no mandatory scheduled visit)</t>
         </is>
       </c>
       <c r="D6" s="6" t="n"/>
@@ -676,7 +676,7 @@
       <c r="B7" s="5" t="n"/>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>18. | Written queries accepted as per tender timeline</t>
+          <t>14.03.2026 14.03, MS Teams, Meeting ID: 436 966 051 957 22, Passcode: o27yw6kA | Written queries accepted as per tender timeline</t>
         </is>
       </c>
       <c r="D7" s="6" t="n"/>
@@ -692,7 +692,7 @@
       <c r="B8" s="5" t="n"/>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Pre-Bid: 18.  →  Bid Due: 02-04-2026 15:00:00  →  Physical Docs: Within 7 days of Bid Due Date  →  Clarifications: 2 Days</t>
+          <t>Pre-Bid: 14.03.2026 14.03, MS Teams, Meeting ID: 436 966 051 957 22, Passcode: o27yw6kA  →  Bid Due: 02-04-2026 15:00:00  →  Physical Docs: Within 7 days of Bid Due Date  →  Clarifications: 2 Days</t>
         </is>
       </c>
       <c r="D8" s="6" t="n"/>
@@ -724,7 +724,7 @@
       <c r="B10" s="5" t="n"/>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Exp: etc. Yrs  |  Financial BEC: Not Applicable (Exempted)</t>
+          <t>Exp: etc. Yrs (Min PO Value: ₹6,214,000.00)  |  Financial BEC: Not Applicable (Exempted)</t>
         </is>
       </c>
       <c r="D10" s="6" t="n"/>
@@ -883,54 +883,54 @@
         </is>
       </c>
       <c r="B21" s="5" t="n"/>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>⚠️ MISSING</t>
-        </is>
-      </c>
-      <c r="D21" s="8" t="n"/>
-      <c r="E21" s="8" t="n"/>
-      <c r="F21" s="8" t="n"/>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>www.GAILonline.com</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="n"/>
+      <c r="E21" s="7" t="n"/>
+      <c r="F21" s="7" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="9" t="inlineStr">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>Bid Due Date and Time</t>
         </is>
       </c>
-      <c r="B22" s="9" t="n"/>
-      <c r="C22" s="10" t="inlineStr">
+      <c r="B22" s="8" t="n"/>
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>02-04-2026 15:00:00</t>
         </is>
       </c>
-      <c r="D22" s="10" t="n"/>
-      <c r="E22" s="10" t="n"/>
-      <c r="F22" s="10" t="n"/>
+      <c r="D22" s="9" t="n"/>
+      <c r="E22" s="9" t="n"/>
+      <c r="F22" s="9" t="n"/>
     </row>
     <row r="23" ht="32" customHeight="1">
-      <c r="A23" s="11" t="inlineStr">
+      <c r="A23" s="10" t="inlineStr">
         <is>
           <t>Recommendation by TE</t>
         </is>
       </c>
-      <c r="B23" s="12" t="inlineStr">
-        <is>
-          <t>⚠️ MISSING</t>
-        </is>
-      </c>
-      <c r="C23" s="11" t="inlineStr">
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Yes — Recommended</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
         <is>
           <t>Reason</t>
         </is>
       </c>
-      <c r="D23" s="13" t="inlineStr">
+      <c r="D23" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="E23" s="13" t="n"/>
-      <c r="F23" s="13" t="n"/>
+      <c r="E23" s="12" t="n"/>
+      <c r="F23" s="12" t="n"/>
     </row>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
@@ -962,9 +962,9 @@
         </is>
       </c>
       <c r="E25" s="6" t="n"/>
-      <c r="F25" s="8" t="inlineStr">
-        <is>
-          <t>⚠️ MISSING</t>
+      <c r="F25" s="12" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
         </is>
       </c>
     </row>
@@ -986,9 +986,9 @@
         </is>
       </c>
       <c r="E26" s="6" t="n"/>
-      <c r="F26" s="8" t="inlineStr">
-        <is>
-          <t>⚠️ MISSING</t>
+      <c r="F26" s="12" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
         </is>
       </c>
     </row>
@@ -1023,9 +1023,9 @@
         </is>
       </c>
       <c r="B28" s="6" t="n"/>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>⚠️ MISSING</t>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>₹0.00</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
@@ -1083,18 +1083,18 @@
           <t>Two Packet Bid</t>
         </is>
       </c>
-      <c r="C30" s="14" t="inlineStr">
+      <c r="C30" s="13" t="inlineStr">
         <is>
           <t>ATC Document Link</t>
         </is>
       </c>
-      <c r="D30" s="14" t="n"/>
-      <c r="E30" s="15" t="inlineStr">
+      <c r="D30" s="13" t="n"/>
+      <c r="E30" s="14" t="inlineStr">
         <is>
           <t>https://fulfilment.gem.gov.in/contract/slafds?fileDownloadPath=SLA_UPLOAD_PATH/2026/Mar/GEM_2026_B_7357339/CLM0010/TENDOC_fd9a524c-f95f-4364-8e261773473753650_gailvizaggem@.pao1.pdf</t>
         </is>
       </c>
-      <c r="F30" s="15" t="n"/>
+      <c r="F30" s="14" t="n"/>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="6" t="inlineStr">
@@ -1102,7 +1102,7 @@
           <t>MAF required</t>
         </is>
       </c>
-      <c r="B31" s="16" t="inlineStr">
+      <c r="B31" s="15" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1112,7 +1112,7 @@
           <t>Delivery Time (Supply/Total)</t>
         </is>
       </c>
-      <c r="D31" s="16" t="inlineStr">
+      <c r="D31" s="6" t="inlineStr">
         <is>
           <t>105 Days</t>
         </is>
@@ -1129,7 +1129,7 @@
       </c>
     </row>
     <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="17" t="inlineStr">
+      <c r="A32" s="16" t="inlineStr">
         <is>
           <t>PBG (in form of)</t>
         </is>
@@ -1144,9 +1144,9 @@
           <t>Payment Terms (Supply)</t>
         </is>
       </c>
-      <c r="D32" s="16" t="inlineStr">
-        <is>
-          <t>70.0</t>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>80%</t>
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr">
@@ -1154,14 +1154,14 @@
           <t>Payment Terms (Installation)</t>
         </is>
       </c>
-      <c r="F32" s="16" t="inlineStr">
-        <is>
-          <t>30.0</t>
+      <c r="F32" s="15" t="inlineStr">
+        <is>
+          <t>20%</t>
         </is>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="17" t="inlineStr">
+      <c r="A33" s="16" t="inlineStr">
         <is>
           <t>SD (in form of)</t>
         </is>
@@ -1186,7 +1186,7 @@
           <t>Max LD %age</t>
         </is>
       </c>
-      <c r="F33" s="16" t="inlineStr">
+      <c r="F33" s="15" t="inlineStr">
         <is>
           <t>5.0</t>
         </is>
@@ -1220,15 +1220,15 @@
           <t>5%</t>
         </is>
       </c>
-      <c r="D35" s="17" t="inlineStr">
+      <c r="D35" s="16" t="inlineStr">
         <is>
           <t>Security Deposit</t>
         </is>
       </c>
-      <c r="E35" s="17" t="n"/>
-      <c r="F35" s="16" t="inlineStr">
-        <is>
-          <t>5.0</t>
+      <c r="E35" s="16" t="n"/>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -1250,25 +1250,25 @@
         </is>
       </c>
       <c r="E36" s="6" t="n"/>
-      <c r="F36" s="8" t="inlineStr">
-        <is>
-          <t>⚠️ MISSING</t>
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="17" t="inlineStr">
+      <c r="A37" s="16" t="inlineStr">
         <is>
           <t>Physical Docs Submission Required</t>
         </is>
       </c>
-      <c r="B37" s="17" t="n"/>
+      <c r="B37" s="16" t="n"/>
       <c r="C37" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D37" s="17" t="inlineStr">
+      <c r="D37" s="16" t="inlineStr">
         <is>
           <t>Physical Docs Submission Deadline</t>
         </is>
@@ -1281,13 +1281,13 @@
       <c r="F37" s="6" t="n"/>
     </row>
     <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="18" t="inlineStr">
+      <c r="A38" s="17" t="inlineStr">
         <is>
           <t>Eligibility Criterion (Years)</t>
         </is>
       </c>
-      <c r="B38" s="18" t="n"/>
-      <c r="C38" s="19" t="inlineStr">
+      <c r="B38" s="17" t="n"/>
+      <c r="C38" s="18" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1307,9 +1307,9 @@
         </is>
       </c>
       <c r="B39" s="6" t="n"/>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>⚠️ MISSING</t>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>₹6,214,000.00</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -1317,12 +1317,12 @@
           <t>Annual Avg Turnover</t>
         </is>
       </c>
-      <c r="E39" s="13" t="inlineStr">
+      <c r="E39" s="12" t="inlineStr">
         <is>
           <t>Not Applicable</t>
         </is>
       </c>
-      <c r="F39" s="13" t="inlineStr">
+      <c r="F39" s="12" t="inlineStr">
         <is>
           <t>₹0.00</t>
         </is>
@@ -1335,9 +1335,9 @@
         </is>
       </c>
       <c r="B40" s="6" t="n"/>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>⚠️ MISSING</t>
+      <c r="C40" s="12" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
@@ -1345,12 +1345,12 @@
           <t>Working Capital</t>
         </is>
       </c>
-      <c r="E40" s="13" t="inlineStr">
+      <c r="E40" s="12" t="inlineStr">
         <is>
           <t>Not Applicable</t>
         </is>
       </c>
-      <c r="F40" s="13" t="inlineStr">
+      <c r="F40" s="12" t="inlineStr">
         <is>
           <t>₹0.00</t>
         </is>
@@ -1363,9 +1363,9 @@
         </is>
       </c>
       <c r="B41" s="6" t="n"/>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>⚠️ MISSING</t>
+      <c r="C41" s="12" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -1373,12 +1373,12 @@
           <t>Net Worth</t>
         </is>
       </c>
-      <c r="E41" s="13" t="inlineStr">
+      <c r="E41" s="12" t="inlineStr">
         <is>
           <t>Not Applicable</t>
         </is>
       </c>
-      <c r="F41" s="13" t="inlineStr">
+      <c r="F41" s="12" t="inlineStr">
         <is>
           <t>₹0.00</t>
         </is>
@@ -1391,9 +1391,9 @@
         </is>
       </c>
       <c r="B42" s="6" t="n"/>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>⚠️ MISSING</t>
+      <c r="C42" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D42" s="6" t="inlineStr">
@@ -1401,12 +1401,12 @@
           <t>Solvency Certificate</t>
         </is>
       </c>
-      <c r="E42" s="13" t="inlineStr">
+      <c r="E42" s="12" t="inlineStr">
         <is>
           <t>Not Applicable</t>
         </is>
       </c>
-      <c r="F42" s="13" t="inlineStr">
+      <c r="F42" s="12" t="inlineStr">
         <is>
           <t>₹0.00</t>
         </is>
@@ -1414,28 +1414,28 @@
     </row>
     <row r="43" ht="15" customHeight="1"/>
     <row r="44" ht="55" customHeight="1">
-      <c r="A44" s="14" t="inlineStr">
+      <c r="A44" s="13" t="inlineStr">
         <is>
           <t>PQC Documents</t>
         </is>
       </c>
-      <c r="B44" s="17" t="inlineStr">
+      <c r="B44" s="16" t="inlineStr">
         <is>
           <t>Document-1, Document-2, Document-3 (Auto attach the documents from PQR dashboard, based on the name selection)</t>
         </is>
       </c>
-      <c r="C44" s="17" t="n"/>
+      <c r="C44" s="16" t="n"/>
       <c r="D44" s="5" t="inlineStr">
         <is>
           <t>Documents for Commercial Eligibility</t>
         </is>
       </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>⚠️ MISSING</t>
-        </is>
-      </c>
-      <c r="F44" s="8" t="n"/>
+      <c r="E44" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F44" s="12" t="n"/>
     </row>
     <row r="45" ht="40" customHeight="1">
       <c r="A45" s="5" t="inlineStr">
@@ -1487,7 +1487,7 @@
           <t>Mobile No.</t>
         </is>
       </c>
-      <c r="F47" s="8" t="inlineStr">
+      <c r="F47" s="19" t="inlineStr">
         <is>
           <t>⚠️ MISSING</t>
         </is>
@@ -1501,7 +1501,7 @@
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>Shri S. Patta</t>
+          <t>Sh. Vishal Kumar</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
-          <t>s.patta@gail.co.in</t>
+          <t>narasingha.rao@gail.co.in</t>
         </is>
       </c>
       <c r="E48" s="6" t="inlineStr">
@@ -1519,9 +1519,9 @@
           <t>Mobile No.</t>
         </is>
       </c>
-      <c r="F48" s="6" t="inlineStr">
-        <is>
-          <t>0891-2513682/9515129199</t>
+      <c r="F48" s="19" t="inlineStr">
+        <is>
+          <t>⚠️ MISSING</t>
         </is>
       </c>
     </row>
@@ -1531,7 +1531,7 @@
           <t>Client Name</t>
         </is>
       </c>
-      <c r="B49" s="13" t="inlineStr">
+      <c r="B49" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1541,7 +1541,7 @@
           <t>Email</t>
         </is>
       </c>
-      <c r="D49" s="13" t="inlineStr">
+      <c r="D49" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1551,7 +1551,7 @@
           <t>Mobile No.</t>
         </is>
       </c>
-      <c r="F49" s="13" t="inlineStr">
+      <c r="F49" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1566,16 +1566,16 @@
       <c r="F50" s="6" t="n"/>
     </row>
     <row r="51" ht="20" customHeight="1">
-      <c r="A51" s="19" t="inlineStr">
+      <c r="A51" s="18" t="inlineStr">
         <is>
           <t>Documents Submitted</t>
         </is>
       </c>
-      <c r="B51" s="19" t="n"/>
-      <c r="C51" s="19" t="n"/>
-      <c r="D51" s="19" t="n"/>
-      <c r="E51" s="19" t="n"/>
-      <c r="F51" s="19" t="n"/>
+      <c r="B51" s="18" t="n"/>
+      <c r="C51" s="18" t="n"/>
+      <c r="D51" s="18" t="n"/>
+      <c r="E51" s="18" t="n"/>
+      <c r="F51" s="18" t="n"/>
     </row>
     <row r="52" ht="20" customHeight="1">
       <c r="A52" s="6" t="inlineStr">
@@ -1647,7 +1647,7 @@
           <t>Doc 7</t>
         </is>
       </c>
-      <c r="B54" s="13" t="inlineStr">
+      <c r="B54" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1657,7 +1657,7 @@
           <t>Doc 8</t>
         </is>
       </c>
-      <c r="D54" s="13" t="inlineStr">
+      <c r="D54" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1667,7 +1667,7 @@
           <t>Doc 9</t>
         </is>
       </c>
-      <c r="F54" s="13" t="inlineStr">
+      <c r="F54" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1680,14 +1680,14 @@
         </is>
       </c>
       <c r="B55" s="6" t="n"/>
-      <c r="C55" s="8" t="inlineStr">
-        <is>
-          <t>⚠️ MISSING</t>
-        </is>
-      </c>
-      <c r="D55" s="8" t="n"/>
-      <c r="E55" s="8" t="n"/>
-      <c r="F55" s="8" t="n"/>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>(s) within Three (03) months (90 Days) from the date of award of GeM contract order/Letter of Intent/Acceptance whichever is issued earlier. The non-completion of supply within stipulated time shall attract Price Reduction Schedule (PRS).</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="n"/>
+      <c r="E55" s="6" t="n"/>
+      <c r="F55" s="6" t="n"/>
     </row>
     <row r="56" ht="20" customHeight="1">
       <c r="A56" s="6" t="inlineStr">
@@ -1711,7 +1711,7 @@
           <t>Courier Provider</t>
         </is>
       </c>
-      <c r="B57" s="8" t="inlineStr">
+      <c r="B57" s="19" t="inlineStr">
         <is>
           <t>⚠️ MISSING</t>
         </is>
@@ -1721,7 +1721,7 @@
           <t>Courier Docket No.</t>
         </is>
       </c>
-      <c r="D57" s="8" t="inlineStr">
+      <c r="D57" s="19" t="inlineStr">
         <is>
           <t>⚠️ MISSING</t>
         </is>
@@ -1731,7 +1731,7 @@
           <t>Delivery time</t>
         </is>
       </c>
-      <c r="F57" s="8" t="inlineStr">
+      <c r="F57" s="19" t="inlineStr">
         <is>
           <t>⚠️ MISSING</t>
         </is>
@@ -1744,7 +1744,7 @@
         </is>
       </c>
       <c r="B58" s="6" t="n"/>
-      <c r="C58" s="8" t="inlineStr">
+      <c r="C58" s="19" t="inlineStr">
         <is>
           <t>⚠️ MISSING</t>
         </is>
@@ -1755,7 +1755,7 @@
         </is>
       </c>
       <c r="E58" s="6" t="n"/>
-      <c r="F58" s="8" t="inlineStr">
+      <c r="F58" s="19" t="inlineStr">
         <is>
           <t>⚠️ MISSING</t>
         </is>
@@ -1801,7 +1801,7 @@
       <c r="E61" s="6" t="n"/>
       <c r="F61" s="6" t="inlineStr">
         <is>
-          <t>Yes | Complete</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1838,7 +1838,7 @@
       <c r="B63" s="6" t="n"/>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>18.</t>
+          <t>14.03.2026 14.03, MS Teams, Meeting ID: 436 966 051 957 22, Passcode: o27yw6kA</t>
         </is>
       </c>
       <c r="D63" s="6" t="n"/>
@@ -1888,14 +1888,14 @@
         </is>
       </c>
       <c r="B67" s="6" t="n"/>
-      <c r="C67" s="13" t="inlineStr">
+      <c r="C67" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="D67" s="13" t="n"/>
-      <c r="E67" s="13" t="n"/>
-      <c r="F67" s="13" t="n"/>
+      <c r="D67" s="12" t="n"/>
+      <c r="E67" s="12" t="n"/>
+      <c r="F67" s="12" t="n"/>
     </row>
     <row r="68" ht="40" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
@@ -1904,14 +1904,14 @@
         </is>
       </c>
       <c r="B68" s="6" t="n"/>
-      <c r="C68" s="13" t="inlineStr">
+      <c r="C68" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="D68" s="13" t="n"/>
-      <c r="E68" s="13" t="n"/>
-      <c r="F68" s="13" t="n"/>
+      <c r="D68" s="12" t="n"/>
+      <c r="E68" s="12" t="n"/>
+      <c r="F68" s="12" t="n"/>
     </row>
     <row r="69" ht="40" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
@@ -1920,14 +1920,14 @@
         </is>
       </c>
       <c r="B69" s="6" t="n"/>
-      <c r="C69" s="8" t="inlineStr">
+      <c r="C69" s="19" t="inlineStr">
         <is>
           <t>⚠️ MISSING</t>
         </is>
       </c>
-      <c r="D69" s="8" t="n"/>
-      <c r="E69" s="8" t="n"/>
-      <c r="F69" s="8" t="n"/>
+      <c r="D69" s="19" t="n"/>
+      <c r="E69" s="19" t="n"/>
+      <c r="F69" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="93">

</xml_diff>